<commit_message>
hoàn thiện giao dịch
</commit_message>
<xml_diff>
--- a/QuanLyChiTieu/Data/Account.xlsx
+++ b/QuanLyChiTieu/Data/Account.xlsx
@@ -46,6 +46,9 @@
   </x:si>
   <x:si>
     <x:t>abcde</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HoaiBao</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1060,6 +1063,14 @@
         <x:v>3</x:v>
       </x:c>
     </x:row>
+    <x:row r="5" spans="1:2">
+      <x:c r="A5" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>